<commit_message>
fix logging and database issue
</commit_message>
<xml_diff>
--- a/data/excels/invoice_details.xlsx
+++ b/data/excels/invoice_details.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Invoice_Master" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Invoices" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -413,216 +413,190 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H5"/>
+  <dimension ref="A1:J4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>Invoice No</t>
+          <t>ID</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>Account No</t>
+          <t>Invoice Number</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
+          <t>Vendor Name</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
           <t>Customer Name</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Total Amount</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>Currency</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>Invoice Date</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>Due Date</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
         <is>
           <t>Payment Status</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>Due Date</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>Shipping Ref</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>Shipping Address</t>
-        </is>
-      </c>
-      <c r="H1" t="inlineStr">
-        <is>
-          <t>Order ID</t>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>Risk Score</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>INV-1001</t>
-        </is>
+      <c r="A2" t="n">
+        <v>1</v>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>ACC-9001</t>
+          <t>INV-1002</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>ABC Corp</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>Paid</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>2025-01-10</t>
-        </is>
+          <t>ABC Technologies Pvt Ltd</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr"/>
+      <c r="E2" t="n">
+        <v>4560</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>SHIP-22</t>
+          <t>USD</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>New York, USA</t>
+          <t>2025-09-10</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>ORD-501</t>
+          <t>2025-10-10</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>Unpaid</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>INV-1002</t>
-        </is>
+      <c r="A3" t="n">
+        <v>2</v>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>ACC-9002</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>XYZ Ltd</t>
-        </is>
-      </c>
+          <t>INV-1001</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr"/>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Pending</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>2025-02-01</t>
-        </is>
+          <t>John Doe</t>
+        </is>
+      </c>
+      <c r="E3" t="n">
+        <v>1250</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>SHIP-45</t>
+          <t>USD</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>London, UK</t>
+          <t>2025-09-15</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>ORD-502</t>
+          <t>2025-10-15</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>Paid</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>LOW</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
+      <c r="A4" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" t="inlineStr">
         <is>
           <t>INV-1003</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>ACC-9003</t>
-        </is>
-      </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Acme Solutions</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>Overdue</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>2025-01-05</t>
-        </is>
+          <t>Robert Industries</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr"/>
+      <c r="E4" t="n">
+        <v>780</v>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>SHIP-78</t>
+          <t>USD</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>Berlin, Germany</t>
+          <t>2025-09-18</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>ORD-503</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>INV1004</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>ACC9004</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>Global Tech Pvt Ltd</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>Paid</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>2025-03-15</t>
-        </is>
-      </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>SHIP-90</t>
-        </is>
-      </c>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>Bangalore, India</t>
-        </is>
-      </c>
-      <c r="H5" t="inlineStr">
-        <is>
-          <t>ORD-504</t>
+          <t>2025-10-18</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>LOW</t>
         </is>
       </c>
     </row>

</xml_diff>